<commit_message>
auto update 2026/04/29 18:00
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -17019,28 +17019,32 @@
       <c r="J222" s="8" t="inlineStr"/>
       <c r="K222" s="8" t="inlineStr">
         <is>
-          <t>2026/05/25</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="L222" s="8" t="inlineStr">
         <is>
-          <t>2026/05/29</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="M222" s="8" t="inlineStr">
         <is>
-          <t>2026/06/20</t>
+          <t>2026/06/05</t>
         </is>
       </c>
       <c r="N222" s="8" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="O222" s="8" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="O222" s="8" t="inlineStr">
+        <is>
+          <t>PCB Layout 中</t>
+        </is>
+      </c>
       <c r="P222" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>1. Schedule: MP pull in 2 weeks 至6/15, DQA測試1week即開始ATS投線, ATS測試同步DQA並行 2. 備料:K級PCB 備料LT 3 Weeks, 5/24 依組裝測試take risk 進行K級備料</t>
         </is>
       </c>
     </row>
@@ -17087,28 +17091,32 @@
       <c r="J223" s="8" t="inlineStr"/>
       <c r="K223" s="8" t="inlineStr">
         <is>
-          <t>2026/05/25</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="L223" s="8" t="inlineStr">
         <is>
-          <t>2026/05/29</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="M223" s="8" t="inlineStr">
         <is>
-          <t>2026/06/20</t>
+          <t>2026/06/05</t>
         </is>
       </c>
       <c r="N223" s="8" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="O223" s="8" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="O223" s="8" t="inlineStr">
+        <is>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
+        </is>
+      </c>
       <c r="P223" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
         </is>
       </c>
     </row>
@@ -17155,28 +17163,32 @@
       <c r="J224" s="8" t="inlineStr"/>
       <c r="K224" s="8" t="inlineStr">
         <is>
-          <t>2026/05/25</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="L224" s="8" t="inlineStr">
         <is>
-          <t>2026/05/29</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="M224" s="8" t="inlineStr">
         <is>
-          <t>2026/06/20</t>
+          <t>2026/06/05</t>
         </is>
       </c>
       <c r="N224" s="8" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="O224" s="8" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="O224" s="8" t="inlineStr">
+        <is>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
+        </is>
+      </c>
       <c r="P224" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
         </is>
       </c>
     </row>
@@ -17223,28 +17235,32 @@
       <c r="J225" s="8" t="inlineStr"/>
       <c r="K225" s="8" t="inlineStr">
         <is>
-          <t>2026/05/25</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="L225" s="8" t="inlineStr">
         <is>
-          <t>2026/05/29</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="M225" s="8" t="inlineStr">
         <is>
-          <t>2026/06/20</t>
+          <t>2026/06/05</t>
         </is>
       </c>
       <c r="N225" s="8" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="O225" s="8" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="O225" s="8" t="inlineStr">
+        <is>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
+        </is>
+      </c>
       <c r="P225" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update 周三 2026/05/06  8:17:21.34
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFC000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00ED7D31"/>
       <sz val="10"/>
     </font>
@@ -118,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -171,25 +176,28 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -5368,7 +5376,7 @@
       <c r="O67" s="8" t="inlineStr"/>
       <c r="P67" s="8" t="inlineStr">
         <is>
-          <t>廠商提供的樣品印刷色彩落差較大，重新打樣中，預計4/30簽樣，5/20進料</t>
+          <t>廠商提供的樣品印刷色彩落差較大，重新打樣中，預計5/4簽樣，5/20進料</t>
         </is>
       </c>
     </row>
@@ -22730,14 +22738,14 @@
           <t>Vector A18 HX A9WHG</t>
         </is>
       </c>
-      <c r="D303" s="9" t="inlineStr">
-        <is>
-          <t>MP</t>
+      <c r="D303" s="11" t="inlineStr">
+        <is>
+          <t>BTO-</t>
         </is>
       </c>
       <c r="E303" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F303" s="8" t="inlineStr">
@@ -22777,12 +22785,12 @@
       </c>
       <c r="M303" s="8" t="inlineStr">
         <is>
-          <t>2025/03/22</t>
+          <t>2025/03/27</t>
         </is>
       </c>
       <c r="N303" s="8" t="inlineStr">
         <is>
-          <t>2025/03/27</t>
+          <t>2025/04/02</t>
         </is>
       </c>
       <c r="O303" s="8" t="inlineStr">
@@ -22790,7 +22798,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P303" s="8" t="inlineStr"/>
+      <c r="P303" s="8" t="inlineStr">
+        <is>
+          <t>BTO未開</t>
+        </is>
+      </c>
     </row>
     <row r="304" hidden="1" outlineLevel="1">
       <c r="A304" s="6" t="n">
@@ -22806,14 +22818,14 @@
           <t>Vector A18 HX A9WHG</t>
         </is>
       </c>
-      <c r="D304" s="11" t="inlineStr">
-        <is>
-          <t>BTO-</t>
+      <c r="D304" s="9" t="inlineStr">
+        <is>
+          <t>MP</t>
         </is>
       </c>
       <c r="E304" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F304" s="8" t="inlineStr">
@@ -22853,24 +22865,20 @@
       </c>
       <c r="M304" s="8" t="inlineStr">
         <is>
+          <t>2025/03/22</t>
+        </is>
+      </c>
+      <c r="N304" s="8" t="inlineStr">
+        <is>
           <t>2025/03/27</t>
         </is>
       </c>
-      <c r="N304" s="8" t="inlineStr">
-        <is>
-          <t>2025/04/02</t>
-        </is>
-      </c>
       <c r="O304" s="8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P304" s="8" t="inlineStr">
-        <is>
-          <t>BTO未開</t>
-        </is>
-      </c>
+      <c r="P304" s="8" t="inlineStr"/>
     </row>
     <row r="305" hidden="1" outlineLevel="1">
       <c r="A305" s="6" t="n">
@@ -22886,14 +22894,14 @@
           <t>Vector A18 HX A9WIG</t>
         </is>
       </c>
-      <c r="D305" s="9" t="inlineStr">
-        <is>
-          <t>MP</t>
+      <c r="D305" s="11" t="inlineStr">
+        <is>
+          <t>BTO-</t>
         </is>
       </c>
       <c r="E305" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F305" s="8" t="inlineStr">
@@ -22933,12 +22941,12 @@
       </c>
       <c r="M305" s="8" t="inlineStr">
         <is>
-          <t>2025/02/19</t>
+          <t>2025/02/16</t>
         </is>
       </c>
       <c r="N305" s="8" t="inlineStr">
         <is>
-          <t>2025/03/14</t>
+          <t>2025/02/28</t>
         </is>
       </c>
       <c r="O305" s="8" t="inlineStr">
@@ -22946,7 +22954,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P305" s="8" t="inlineStr"/>
+      <c r="P305" s="8" t="inlineStr">
+        <is>
+          <t>BTO未開</t>
+        </is>
+      </c>
     </row>
     <row r="306" hidden="1" outlineLevel="1">
       <c r="A306" s="6" t="n">
@@ -22962,14 +22974,14 @@
           <t>Vector A18 HX A9WIG</t>
         </is>
       </c>
-      <c r="D306" s="11" t="inlineStr">
-        <is>
-          <t>BTO-</t>
+      <c r="D306" s="9" t="inlineStr">
+        <is>
+          <t>MP</t>
         </is>
       </c>
       <c r="E306" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F306" s="8" t="inlineStr">
@@ -23009,12 +23021,12 @@
       </c>
       <c r="M306" s="8" t="inlineStr">
         <is>
-          <t>2025/02/16</t>
+          <t>2025/02/19</t>
         </is>
       </c>
       <c r="N306" s="8" t="inlineStr">
         <is>
-          <t>2025/02/28</t>
+          <t>2025/03/14</t>
         </is>
       </c>
       <c r="O306" s="8" t="inlineStr">
@@ -23022,11 +23034,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P306" s="8" t="inlineStr">
-        <is>
-          <t>BTO未開</t>
-        </is>
-      </c>
+      <c r="P306" s="8" t="inlineStr"/>
     </row>
     <row r="307" hidden="1" outlineLevel="1">
       <c r="A307" s="6" t="n">
@@ -23049,7 +23057,7 @@
       </c>
       <c r="E307" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F307" s="8" t="inlineStr">
@@ -23129,7 +23137,7 @@
       </c>
       <c r="E308" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F308" s="8" t="inlineStr">
@@ -28086,14 +28094,14 @@
           <t>Cyborg A15 AI+ B3HWGKG</t>
         </is>
       </c>
-      <c r="D375" s="11" t="inlineStr">
-        <is>
-          <t>BTO-</t>
+      <c r="D375" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E375" s="8" t="inlineStr">
         <is>
-          <t>KRK-H 45W</t>
+          <t>HWK 45W</t>
         </is>
       </c>
       <c r="F375" s="8" t="inlineStr">
@@ -28112,34 +28120,26 @@
         </is>
       </c>
       <c r="I375" s="8" t="inlineStr"/>
-      <c r="J375" s="8" t="inlineStr">
-        <is>
-          <t>2025/02/27</t>
-        </is>
-      </c>
-      <c r="K375" s="8" t="inlineStr">
-        <is>
-          <t>2025/04/15</t>
-        </is>
-      </c>
+      <c r="J375" s="8" t="inlineStr"/>
+      <c r="K375" s="8" t="inlineStr"/>
       <c r="L375" s="8" t="inlineStr">
         <is>
-          <t>2025/04/10</t>
+          <t>2025/06/10</t>
         </is>
       </c>
       <c r="M375" s="8" t="inlineStr">
         <is>
-          <t>2025/06/11</t>
+          <t>2025/08/12</t>
         </is>
       </c>
       <c r="N375" s="8" t="inlineStr">
         <is>
-          <t>2025/06/21</t>
+          <t>2025/08/18</t>
         </is>
       </c>
       <c r="O375" s="8" t="inlineStr">
         <is>
-          <t>BTO 未開放</t>
+          <t>165HZ panel 交期8/E或者9/B，業務急單36台 assy@8/12，入庫：8/18</t>
         </is>
       </c>
       <c r="P375" s="8" t="inlineStr">
@@ -28162,14 +28162,14 @@
           <t>Cyborg A15 AI+ B3HWGKG</t>
         </is>
       </c>
-      <c r="D376" s="12" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="D376" s="11" t="inlineStr">
+        <is>
+          <t>BTO-</t>
         </is>
       </c>
       <c r="E376" s="8" t="inlineStr">
         <is>
-          <t>HWK 45W</t>
+          <t>KRK-H 45W</t>
         </is>
       </c>
       <c r="F376" s="8" t="inlineStr">
@@ -28188,26 +28188,34 @@
         </is>
       </c>
       <c r="I376" s="8" t="inlineStr"/>
-      <c r="J376" s="8" t="inlineStr"/>
-      <c r="K376" s="8" t="inlineStr"/>
+      <c r="J376" s="8" t="inlineStr">
+        <is>
+          <t>2025/02/27</t>
+        </is>
+      </c>
+      <c r="K376" s="8" t="inlineStr">
+        <is>
+          <t>2025/04/15</t>
+        </is>
+      </c>
       <c r="L376" s="8" t="inlineStr">
         <is>
-          <t>2025/06/10</t>
+          <t>2025/04/10</t>
         </is>
       </c>
       <c r="M376" s="8" t="inlineStr">
         <is>
-          <t>2025/08/12</t>
+          <t>2025/06/11</t>
         </is>
       </c>
       <c r="N376" s="8" t="inlineStr">
         <is>
-          <t>2025/08/18</t>
+          <t>2025/06/21</t>
         </is>
       </c>
       <c r="O376" s="8" t="inlineStr">
         <is>
-          <t>165HZ panel 交期8/E或者9/B，業務急單36台 assy@8/12，入庫：8/18</t>
+          <t>BTO 未開放</t>
         </is>
       </c>
       <c r="P376" s="8" t="inlineStr">
@@ -29710,9 +29718,9 @@
           <t>Cyborg 15 C13WEO</t>
         </is>
       </c>
-      <c r="D397" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D397" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E397" s="8" t="inlineStr">
@@ -29759,7 +29767,7 @@
       </c>
       <c r="O397" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>預計5/8 ATS C/R@26PN045660*50pcs</t>
         </is>
       </c>
       <c r="P397" s="8" t="inlineStr">
@@ -29782,9 +29790,9 @@
           <t>Cyborg 15 C13WFO</t>
         </is>
       </c>
-      <c r="D398" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D398" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E398" s="8" t="inlineStr">
@@ -29831,7 +29839,7 @@
       </c>
       <c r="O398" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>同Cyborg 15 C13WEO</t>
         </is>
       </c>
       <c r="P398" s="8" t="inlineStr">
@@ -29854,9 +29862,9 @@
           <t>Cyborg 15 C2WEO</t>
         </is>
       </c>
-      <c r="D399" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D399" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E399" s="8" t="inlineStr">
@@ -29903,12 +29911,12 @@
       </c>
       <c r="O399" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
       <c r="P399" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
     </row>
@@ -29926,9 +29934,9 @@
           <t>Cyborg 15 C2WFO</t>
         </is>
       </c>
-      <c r="D400" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D400" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E400" s="8" t="inlineStr">
@@ -29975,12 +29983,12 @@
       </c>
       <c r="O400" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
       <c r="P400" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
     </row>
@@ -29998,9 +30006,9 @@
           <t>Cyborg 15 Max C13WEO</t>
         </is>
       </c>
-      <c r="D401" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D401" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E401" s="8" t="inlineStr">
@@ -30047,7 +30055,7 @@
       </c>
       <c r="O401" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>同Cyborg 15 C13WEO</t>
         </is>
       </c>
       <c r="P401" s="8" t="inlineStr">
@@ -30070,9 +30078,9 @@
           <t>Cyborg 15 Max C13WFO</t>
         </is>
       </c>
-      <c r="D402" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D402" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E402" s="8" t="inlineStr">
@@ -30119,7 +30127,7 @@
       </c>
       <c r="O402" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>同Cyborg 15 C13WEO</t>
         </is>
       </c>
       <c r="P402" s="8" t="inlineStr">
@@ -30142,9 +30150,9 @@
           <t>Cyborg 15 Max C13WGO</t>
         </is>
       </c>
-      <c r="D403" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D403" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E403" s="8" t="inlineStr">
@@ -30191,7 +30199,7 @@
       </c>
       <c r="O403" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>同Cyborg 15 C13WEO</t>
         </is>
       </c>
       <c r="P403" s="8" t="inlineStr">
@@ -30214,9 +30222,9 @@
           <t>Cyborg 15 Max C2WEO</t>
         </is>
       </c>
-      <c r="D404" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D404" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E404" s="8" t="inlineStr">
@@ -30263,12 +30271,12 @@
       </c>
       <c r="O404" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
       <c r="P404" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
     </row>
@@ -30286,9 +30294,9 @@
           <t>Cyborg 15 Max C2WFO</t>
         </is>
       </c>
-      <c r="D405" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D405" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E405" s="8" t="inlineStr">
@@ -30335,12 +30343,12 @@
       </c>
       <c r="O405" s="8" t="inlineStr">
         <is>
-          <t>Status the same Cyborg 15 Max C2WGO</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
       <c r="P405" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
     </row>
@@ -30358,9 +30366,9 @@
           <t>Cyborg 15 Max C2WGO</t>
         </is>
       </c>
-      <c r="D406" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D406" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E406" s="8" t="inlineStr">
@@ -30407,12 +30415,12 @@
       </c>
       <c r="O406" s="8" t="inlineStr">
         <is>
-          <t>MVT 測試中</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
       <c r="P406" s="8" t="inlineStr">
         <is>
-          <t>預計5/6 ATS C/R RPL-H, 目前兩個問題請RDSW儘速釐清 1.使用網易雲客戶端播放音樂，幾率性出現PO音 2. DC下透過瀏覽器播放線上影片,播放一會影片會卡頓</t>
+          <t>待業務通知開BTO</t>
         </is>
       </c>
     </row>
@@ -30499,12 +30507,12 @@
       </c>
       <c r="C408" s="4" t="inlineStr">
         <is>
-          <t>Cyborg A15 C1WE</t>
-        </is>
-      </c>
-      <c r="D408" s="18" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Cyborg A15 Max C1WE</t>
+        </is>
+      </c>
+      <c r="D408" s="19" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E408" s="4" t="inlineStr">
@@ -30524,7 +30532,7 @@
       </c>
       <c r="H408" s="4" t="inlineStr">
         <is>
-          <t>2025/10/17</t>
+          <t>2025/10/03</t>
         </is>
       </c>
       <c r="I408" s="4" t="inlineStr">
@@ -30545,12 +30553,12 @@
       </c>
       <c r="M408" s="4" t="inlineStr">
         <is>
-          <t>2026/06/26</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="N408" s="4" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O408" s="4" t="inlineStr">
@@ -30575,12 +30583,12 @@
       </c>
       <c r="C409" s="8" t="inlineStr">
         <is>
-          <t>Cyborg A15 C1WF</t>
-        </is>
-      </c>
-      <c r="D409" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Cyborg A15 Max C1WF</t>
+        </is>
+      </c>
+      <c r="D409" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E409" s="8" t="inlineStr">
@@ -30600,7 +30608,7 @@
       </c>
       <c r="H409" s="8" t="inlineStr">
         <is>
-          <t>2025/10/17</t>
+          <t>2025/10/03</t>
         </is>
       </c>
       <c r="I409" s="8" t="inlineStr">
@@ -30621,12 +30629,12 @@
       </c>
       <c r="M409" s="8" t="inlineStr">
         <is>
-          <t>2026/06/26</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="N409" s="8" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O409" s="8" t="inlineStr">
@@ -30651,12 +30659,12 @@
       </c>
       <c r="C410" s="8" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1WE</t>
-        </is>
-      </c>
-      <c r="D410" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Cyborg A15 Max C1WG</t>
+        </is>
+      </c>
+      <c r="D410" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E410" s="8" t="inlineStr">
@@ -30666,7 +30674,7 @@
       </c>
       <c r="F410" s="8" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G410" s="8" t="inlineStr">
@@ -30697,22 +30705,22 @@
       </c>
       <c r="M410" s="8" t="inlineStr">
         <is>
-          <t>2026/06/26</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="N410" s="8" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O410" s="8" t="inlineStr">
         <is>
-          <t>同Cyborg A15 Max C1WG</t>
+          <t>暫定 5/20 ATS Assy, 5/30 2nd MP</t>
         </is>
       </c>
       <c r="P410" s="8" t="inlineStr">
         <is>
-          <t>同Cyborg A15 Max C1WG</t>
+          <t>4/30備料會議討論後暫定 5/20 ATS Assy, 5/30 2nd MP,最終 ATS 時程將依物料齊套狀況再行調整,目前已知缺料瓶頸為 KB shielding,已重新開 BTO,請 Vincent/Eva 協助通知業務儘速下單入系統,以利物管確認是否仍有其他缺料項目</t>
         </is>
       </c>
     </row>
@@ -30727,12 +30735,12 @@
       </c>
       <c r="C411" s="8" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1WF</t>
-        </is>
-      </c>
-      <c r="D411" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Cyborg A15 C1WE</t>
+        </is>
+      </c>
+      <c r="D411" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E411" s="8" t="inlineStr">
@@ -30742,7 +30750,7 @@
       </c>
       <c r="F411" s="8" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G411" s="8" t="inlineStr">
@@ -30752,7 +30760,7 @@
       </c>
       <c r="H411" s="8" t="inlineStr">
         <is>
-          <t>2025/10/03</t>
+          <t>2025/10/17</t>
         </is>
       </c>
       <c r="I411" s="8" t="inlineStr">
@@ -30773,12 +30781,12 @@
       </c>
       <c r="M411" s="8" t="inlineStr">
         <is>
-          <t>2026/06/26</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="N411" s="8" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O411" s="8" t="inlineStr">
@@ -30803,12 +30811,12 @@
       </c>
       <c r="C412" s="8" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1WG</t>
-        </is>
-      </c>
-      <c r="D412" s="14" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Cyborg A15 C1WF</t>
+        </is>
+      </c>
+      <c r="D412" s="18" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E412" s="8" t="inlineStr">
@@ -30818,7 +30826,7 @@
       </c>
       <c r="F412" s="8" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G412" s="8" t="inlineStr">
@@ -30828,7 +30836,7 @@
       </c>
       <c r="H412" s="8" t="inlineStr">
         <is>
-          <t>2025/10/03</t>
+          <t>2025/10/17</t>
         </is>
       </c>
       <c r="I412" s="8" t="inlineStr">
@@ -30849,22 +30857,22 @@
       </c>
       <c r="M412" s="8" t="inlineStr">
         <is>
-          <t>2026/06/26</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="N412" s="8" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O412" s="8" t="inlineStr">
         <is>
-          <t>依CPU WW 26進廠進行 ATS</t>
+          <t>同Cyborg A15 Max C1WG</t>
         </is>
       </c>
       <c r="P412" s="8" t="inlineStr">
         <is>
-          <t>採購l持續協助pull in CPU交期, 如有提前會更新ATS時間</t>
+          <t>同Cyborg A15 Max C1WG</t>
         </is>
       </c>
     </row>
@@ -37125,7 +37133,7 @@
       </c>
       <c r="E498" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX refresh 55W</t>
+          <t>ARL-HX 55W</t>
         </is>
       </c>
       <c r="F498" s="8" t="inlineStr">
@@ -37144,25 +37152,25 @@
         </is>
       </c>
       <c r="I498" s="8" t="inlineStr"/>
-      <c r="J498" s="8" t="inlineStr"/>
-      <c r="K498" s="8" t="inlineStr">
-        <is>
-          <t>2025/12/19</t>
-        </is>
-      </c>
+      <c r="J498" s="8" t="inlineStr">
+        <is>
+          <t>2025/10/21</t>
+        </is>
+      </c>
+      <c r="K498" s="8" t="inlineStr"/>
       <c r="L498" s="8" t="inlineStr">
         <is>
-          <t>2026/01/05</t>
+          <t>2026/01/13</t>
         </is>
       </c>
       <c r="M498" s="8" t="inlineStr">
         <is>
-          <t>2026/03/09</t>
+          <t>2026/02/02</t>
         </is>
       </c>
       <c r="N498" s="8" t="inlineStr">
         <is>
-          <t>2026/03/21</t>
+          <t>2026/02/26</t>
         </is>
       </c>
       <c r="O498" s="8" t="inlineStr">
@@ -37197,7 +37205,7 @@
       </c>
       <c r="E499" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX 55W</t>
+          <t>ARL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F499" s="8" t="inlineStr">
@@ -37216,25 +37224,25 @@
         </is>
       </c>
       <c r="I499" s="8" t="inlineStr"/>
-      <c r="J499" s="8" t="inlineStr">
-        <is>
-          <t>2025/10/21</t>
-        </is>
-      </c>
-      <c r="K499" s="8" t="inlineStr"/>
+      <c r="J499" s="8" t="inlineStr"/>
+      <c r="K499" s="8" t="inlineStr">
+        <is>
+          <t>2025/12/19</t>
+        </is>
+      </c>
       <c r="L499" s="8" t="inlineStr">
         <is>
-          <t>2026/01/13</t>
+          <t>2026/01/05</t>
         </is>
       </c>
       <c r="M499" s="8" t="inlineStr">
         <is>
-          <t>2026/02/02</t>
+          <t>2026/03/09</t>
         </is>
       </c>
       <c r="N499" s="8" t="inlineStr">
         <is>
-          <t>2026/02/26</t>
+          <t>2026/03/21</t>
         </is>
       </c>
       <c r="O499" s="8" t="inlineStr">
@@ -37269,7 +37277,7 @@
       </c>
       <c r="E500" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX 55W</t>
+          <t>ARL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F500" s="8" t="inlineStr">
@@ -37287,17 +37295,13 @@
           <t>2025/06/25</t>
         </is>
       </c>
-      <c r="I500" s="8" t="inlineStr">
-        <is>
-          <t>2025/08/12</t>
-        </is>
-      </c>
-      <c r="J500" s="8" t="inlineStr">
-        <is>
-          <t>2025/10/21</t>
-        </is>
-      </c>
-      <c r="K500" s="8" t="inlineStr"/>
+      <c r="I500" s="8" t="inlineStr"/>
+      <c r="J500" s="8" t="inlineStr"/>
+      <c r="K500" s="8" t="inlineStr">
+        <is>
+          <t>2025/12/06</t>
+        </is>
+      </c>
       <c r="L500" s="8" t="inlineStr">
         <is>
           <t>2026/01/05</t>
@@ -37305,12 +37309,12 @@
       </c>
       <c r="M500" s="8" t="inlineStr">
         <is>
-          <t>2026/02/28</t>
+          <t>2026/03/09</t>
         </is>
       </c>
       <c r="N500" s="8" t="inlineStr">
         <is>
-          <t>2026/03/06</t>
+          <t>2026/03/21</t>
         </is>
       </c>
       <c r="O500" s="8" t="inlineStr">
@@ -37345,7 +37349,7 @@
       </c>
       <c r="E501" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX refresh 55W</t>
+          <t>ARL-HX 55W</t>
         </is>
       </c>
       <c r="F501" s="8" t="inlineStr">
@@ -37363,13 +37367,17 @@
           <t>2025/06/25</t>
         </is>
       </c>
-      <c r="I501" s="8" t="inlineStr"/>
-      <c r="J501" s="8" t="inlineStr"/>
-      <c r="K501" s="8" t="inlineStr">
-        <is>
-          <t>2025/12/06</t>
-        </is>
-      </c>
+      <c r="I501" s="8" t="inlineStr">
+        <is>
+          <t>2025/08/12</t>
+        </is>
+      </c>
+      <c r="J501" s="8" t="inlineStr">
+        <is>
+          <t>2025/10/21</t>
+        </is>
+      </c>
+      <c r="K501" s="8" t="inlineStr"/>
       <c r="L501" s="8" t="inlineStr">
         <is>
           <t>2026/01/05</t>
@@ -37377,12 +37385,12 @@
       </c>
       <c r="M501" s="8" t="inlineStr">
         <is>
-          <t>2026/03/09</t>
+          <t>2026/02/28</t>
         </is>
       </c>
       <c r="N501" s="8" t="inlineStr">
         <is>
-          <t>2026/03/21</t>
+          <t>2026/03/06</t>
         </is>
       </c>
       <c r="O501" s="8" t="inlineStr">
@@ -37557,7 +37565,7 @@
       </c>
       <c r="E504" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX refresh 55W</t>
+          <t>ARL-HX 55W</t>
         </is>
       </c>
       <c r="F504" s="8" t="inlineStr">
@@ -37577,20 +37585,24 @@
       </c>
       <c r="I504" s="8" t="inlineStr"/>
       <c r="J504" s="8" t="inlineStr"/>
-      <c r="K504" s="8" t="inlineStr"/>
+      <c r="K504" s="8" t="inlineStr">
+        <is>
+          <t>2026/01/12</t>
+        </is>
+      </c>
       <c r="L504" s="8" t="inlineStr">
         <is>
-          <t>2026/01/12</t>
+          <t>2026/01/05</t>
         </is>
       </c>
       <c r="M504" s="8" t="inlineStr">
         <is>
-          <t>2026/03/09</t>
+          <t>2026/02/28</t>
         </is>
       </c>
       <c r="N504" s="8" t="inlineStr">
         <is>
-          <t>2026/03/21</t>
+          <t>2026/03/13</t>
         </is>
       </c>
       <c r="O504" s="8" t="inlineStr">
@@ -37625,7 +37637,7 @@
       </c>
       <c r="E505" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX 55W</t>
+          <t>ARL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F505" s="8" t="inlineStr">
@@ -37645,24 +37657,20 @@
       </c>
       <c r="I505" s="8" t="inlineStr"/>
       <c r="J505" s="8" t="inlineStr"/>
-      <c r="K505" s="8" t="inlineStr">
+      <c r="K505" s="8" t="inlineStr"/>
+      <c r="L505" s="8" t="inlineStr">
         <is>
           <t>2026/01/12</t>
         </is>
       </c>
-      <c r="L505" s="8" t="inlineStr">
-        <is>
-          <t>2026/01/05</t>
-        </is>
-      </c>
       <c r="M505" s="8" t="inlineStr">
         <is>
-          <t>2026/02/28</t>
+          <t>2026/03/09</t>
         </is>
       </c>
       <c r="N505" s="8" t="inlineStr">
         <is>
-          <t>2026/03/13</t>
+          <t>2026/03/21</t>
         </is>
       </c>
       <c r="O505" s="8" t="inlineStr">
@@ -37697,7 +37705,7 @@
       </c>
       <c r="E506" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX 55W</t>
+          <t>ARL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F506" s="8" t="inlineStr">
@@ -37765,7 +37773,7 @@
       </c>
       <c r="E507" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX refresh 55W</t>
+          <t>ARL-HX 55W</t>
         </is>
       </c>
       <c r="F507" s="8" t="inlineStr">
@@ -38721,7 +38729,7 @@
       </c>
       <c r="E520" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX 55W</t>
+          <t>ARL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F520" s="8" t="inlineStr">
@@ -38797,7 +38805,7 @@
       </c>
       <c r="E521" s="8" t="inlineStr">
         <is>
-          <t>ARL-HX refresh 55W</t>
+          <t>ARL-HX 55W</t>
         </is>
       </c>
       <c r="F521" s="8" t="inlineStr">
@@ -39525,10 +39533,14 @@
           <t>2026/06/09</t>
         </is>
       </c>
-      <c r="O530" s="8" t="inlineStr"/>
+      <c r="O530" s="8" t="inlineStr">
+        <is>
+          <t>无需求，暂未开放BTO</t>
+        </is>
+      </c>
       <c r="P530" s="8" t="inlineStr">
         <is>
-          <t>follow Crosshair 16 HX MLG Edition E14WGK</t>
+          <t>follow RTX5060</t>
         </is>
       </c>
     </row>
@@ -39596,7 +39608,7 @@
       <c r="O531" s="8" t="inlineStr"/>
       <c r="P531" s="8" t="inlineStr">
         <is>
-          <t>follow Crosshair 16 HX MLG Edition E14WGK</t>
+          <t>1. KB白色key cap QUV test 待5/4確認結果後更新KB MP物料交期 2. 2653 MLG A &amp; B side膠粒預計交期@5/11，成型307 預計5/21 for MVT 3.Take risk , 首批成型3K套 4.5/28 MVT測試與ATS同步進行，TTM pull in至 6/9 5.MVT 驗證 , if issue , waive or 增加輔料for short term</t>
         </is>
       </c>
     </row>
@@ -39663,12 +39675,12 @@
       </c>
       <c r="O532" s="8" t="inlineStr">
         <is>
-          <t>報價單未確定，BTO暫未開放</t>
+          <t>无需求，暂未开放BTO</t>
         </is>
       </c>
       <c r="P532" s="8" t="inlineStr">
         <is>
-          <t>1. 報價單未確定，BTO暫未開放 2. 2653 MLG A &amp; B side膠粒預計交期@5/11，成型307 預計5/21 for MVT 3.Take risk , 首批成型3K套 4.5/28 MVT測試與ATS同步進行，TTM pull in至 6/9 5.MVT 驗證 , if issue , waive or 增加輔料for short term</t>
+          <t>follow RTX 5060</t>
         </is>
       </c>
     </row>
@@ -39929,7 +39941,7 @@
       </c>
       <c r="E536" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F536" s="8" t="inlineStr">
@@ -39997,7 +40009,7 @@
       </c>
       <c r="E537" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F537" s="8" t="inlineStr">
@@ -40065,7 +40077,7 @@
       </c>
       <c r="E538" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F538" s="8" t="inlineStr">
@@ -40133,7 +40145,7 @@
       </c>
       <c r="E539" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F539" s="8" t="inlineStr">
@@ -40201,7 +40213,7 @@
       </c>
       <c r="E540" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F540" s="8" t="inlineStr">
@@ -40269,7 +40281,7 @@
       </c>
       <c r="E541" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F541" s="8" t="inlineStr">
@@ -40406,9 +40418,9 @@
           <t>Crosshair A16 HX E8WFK</t>
         </is>
       </c>
-      <c r="D543" s="19" t="inlineStr">
-        <is>
-          <t>ATS</t>
+      <c r="D543" s="9" t="inlineStr">
+        <is>
+          <t>MP</t>
         </is>
       </c>
       <c r="E543" s="8" t="inlineStr">
@@ -40486,9 +40498,9 @@
           <t>Crosshair A16 HX E8WGK</t>
         </is>
       </c>
-      <c r="D544" s="19" t="inlineStr">
-        <is>
-          <t>ATS</t>
+      <c r="D544" s="9" t="inlineStr">
+        <is>
+          <t>MP</t>
         </is>
       </c>
       <c r="E544" s="8" t="inlineStr">
@@ -40610,12 +40622,12 @@
       </c>
       <c r="N545" s="8" t="inlineStr">
         <is>
-          <t>2026/05/29</t>
+          <t>2026/05/25</t>
         </is>
       </c>
       <c r="O545" s="8" t="inlineStr">
         <is>
-          <t>MVT 測試中</t>
+          <t>MVT 測試中,ATS 走C/R</t>
         </is>
       </c>
       <c r="P545" s="8" t="inlineStr">
@@ -40645,7 +40657,7 @@
       </c>
       <c r="E546" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F546" s="8" t="inlineStr">
@@ -40685,11 +40697,7 @@
           <t>2026/06/28</t>
         </is>
       </c>
-      <c r="O546" s="8" t="inlineStr">
-        <is>
-          <t>2026/1/12 會議通知pending FRG</t>
-        </is>
-      </c>
+      <c r="O546" s="8" t="inlineStr"/>
       <c r="P546" s="8" t="inlineStr">
         <is>
           <t>NA</t>
@@ -40717,7 +40725,7 @@
       </c>
       <c r="E547" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F547" s="8" t="inlineStr">
@@ -40757,7 +40765,11 @@
           <t>2026/06/28</t>
         </is>
       </c>
-      <c r="O547" s="8" t="inlineStr"/>
+      <c r="O547" s="8" t="inlineStr">
+        <is>
+          <t>2026/1/12 會議通知pending FRG</t>
+        </is>
+      </c>
       <c r="P547" s="8" t="inlineStr">
         <is>
           <t>NA</t>
@@ -41421,7 +41433,7 @@
       </c>
       <c r="E557" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F557" s="8" t="inlineStr">
@@ -41489,7 +41501,7 @@
       </c>
       <c r="E558" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F558" s="8" t="inlineStr">
@@ -41557,7 +41569,7 @@
       </c>
       <c r="E559" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F559" s="8" t="inlineStr">
@@ -41625,7 +41637,7 @@
       </c>
       <c r="E560" s="8" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F560" s="8" t="inlineStr">
@@ -42696,7 +42708,7 @@
       </c>
       <c r="D574" s="20" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Study</t>
         </is>
       </c>
       <c r="E574" s="4" t="inlineStr">
@@ -42750,7 +42762,11 @@
         </is>
       </c>
       <c r="O574" s="4" t="inlineStr"/>
-      <c r="P574" s="4" t="inlineStr"/>
+      <c r="P574" s="4" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
     </row>
     <row r="575" ht="20" customHeight="1">
       <c r="A575" s="2" t="n">
@@ -44206,7 +44222,7 @@
           <t>Katana 15 HX C14WEK</t>
         </is>
       </c>
-      <c r="D593" s="20" t="inlineStr">
+      <c r="D593" s="21" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -44259,12 +44275,12 @@
       </c>
       <c r="O593" s="4" t="inlineStr">
         <is>
-          <t>follow Katana 15 HX C14WFK</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
       <c r="P593" s="4" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
     </row>
@@ -44335,12 +44351,12 @@
       </c>
       <c r="O594" s="8" t="inlineStr">
         <is>
-          <t>follow Katana 15 HX C14WFK</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
       <c r="P594" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
     </row>
@@ -44411,12 +44427,12 @@
       </c>
       <c r="O595" s="8" t="inlineStr">
         <is>
-          <t>follow Katana 15 HX C14WFK</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
       <c r="P595" s="8" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>同Katana 15 HX C14WGXK</t>
         </is>
       </c>
     </row>
@@ -44492,7 +44508,7 @@
       </c>
       <c r="P596" s="8" t="inlineStr">
         <is>
-          <t>1.Color Plan未定案影響開模,schedule待定案後確認 2.進入MVT 前先確認業務是否有GDDR7 8GB的出貨需求, 若有, 則需額外增加 MVT 機台給 RD 測試。</t>
+          <t>15T3 時程相當緊急,組裝僅有一次MVT,之後就進入ATS,由於系列設計尚未定案，team member 目前無法確認開模與修模方向,且部分模具與 15T1/15T2 共用,仍需協調可挪用時程,請 ID/SPM 務必於 5/5 前完成定案.</t>
         </is>
       </c>
     </row>
@@ -47530,7 +47546,7 @@
           <t>Prestige N14 AI+ D1M</t>
         </is>
       </c>
-      <c r="D637" s="21" t="inlineStr">
+      <c r="D637" s="22" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -48758,7 +48774,7 @@
           <t>Prestige N16 Flip AI+</t>
         </is>
       </c>
-      <c r="D653" s="21" t="inlineStr">
+      <c r="D653" s="22" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -48820,7 +48836,7 @@
       </c>
       <c r="P653" s="4" t="inlineStr">
         <is>
-          <t>1.Stop code 0x101問題，依Incyde BIOS修改後，有降低發生機率，主要影響long run測試，NV與MTK確認patch中，待更新結果。 2.MSFT 4/7 release OS WIR 3E，insyde 4/9 release BIOS for BSP PS drop 0.3，須請RD協助於4/10前更新BIOS與HDI 3.4/8會議更新Workshop2執行config如下 Pre-work BSP:6.0.6 Bug verification:BSP PS drop 0.3 +OS WIR 3E</t>
+          <t>1.因應PWR要求重工電阻，去解系統無法跑重載的問題，另衍生128GB SKU會當機的issue，PWR初步分析為PWM IC的來料問題，廠商4/30下午重工實驗中，需over night確認實驗結果後。 2.原預計5/4進CER，image版本已確認為2.9版，BIOS為43版，但因前項問題仍待釐清，待RD釐清後，與MSFT確認作法 3.Battery life a)因目前有PWM IC來料問題，待釐清並重工後，DQA會重新開始測試。 b) power break down，待廠商提供相關FW更新後，由HW與廠商持續釐清中。</t>
         </is>
       </c>
     </row>
@@ -48838,7 +48854,7 @@
           <t>Prestige N16 AI+</t>
         </is>
       </c>
-      <c r="D654" s="22" t="inlineStr">
+      <c r="D654" s="23" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -48900,7 +48916,7 @@
       </c>
       <c r="P654" s="8" t="inlineStr">
         <is>
-          <t>1.Stop code 0x101問題，依Incyde BIOS修改後，有降低發生機率，主要影響long run測試，NV與MTK確認patch中，待更新結果。 2.MSFT 4/7 release OS WIR 3E，insyde 4/9 release BIOS for BSP PS drop 0.3，須請RD協助於4/10前更新BIOS與HDI 3.4/8會議更新Workshop2執行config如下 Pre-work BSP:6.0.6 Bug verification:BSP PS drop 0.3 +OS WIR 3E</t>
+          <t>1.因應PWR要求重工電阻，去解系統無法跑重載的問題，另衍生128GB SKU會當機的issue，PWR初步分析為PWM IC的來料問題，廠商4/30下午重工實驗中，需over night確認實驗結果後。 2.原預計5/4進CER，image版本已確認為2.9版，BIOS為43版，但因前項問題仍待釐清，待RD釐清後，與MSFT確認作法 3.Battery life a)因目前有PWM IC來料問題，待釐清並重工後，DQA會重新開始測試。 b) power break down，待廠商提供相關FW更新後，由HW與廠商持續釐清中。</t>
         </is>
       </c>
     </row>
@@ -49230,7 +49246,7 @@
           <t>Prestige N16 AI+ C1M</t>
         </is>
       </c>
-      <c r="D659" s="21" t="inlineStr">
+      <c r="D659" s="22" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -49287,7 +49303,7 @@
       </c>
       <c r="O659" s="4" t="inlineStr">
         <is>
-          <t>EVT 機台預計4/24調撥回台給RD驗證, 預計 6/5 ver. 1.0  出圖</t>
+          <t>EVT 機台於4/28已經抵台陸續分發給RD 驗證,並且Week 5/4 當周分別寄送給NV 各辦公室測試</t>
         </is>
       </c>
       <c r="P659" s="4" t="inlineStr">
@@ -51046,7 +51062,7 @@
           <t>Modern 14 H1M</t>
         </is>
       </c>
-      <c r="D684" s="18" t="inlineStr">
+      <c r="D684" s="24" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
@@ -51104,7 +51120,7 @@
       </c>
       <c r="P684" s="4" t="inlineStr">
         <is>
-          <t>備料：因鍵盤絲印需要廠商印刷，齊料時間5/15,持續 Tracking 物料交期</t>
+          <t>物料 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  認證  泰國 需業務push進口商提供認證資料,資料Ready後+3W PIC: Sales   馬來西亞 進口商WIFI 模組證書失效需盡快提供認證資料, 資料Ready後+5W PIC: Sale</t>
         </is>
       </c>
     </row>
@@ -51165,12 +51181,12 @@
       </c>
       <c r="M685" s="8" t="inlineStr">
         <is>
-          <t>2026/05/09</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="N685" s="8" t="inlineStr">
         <is>
-          <t>2026/05/21</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O685" s="8" t="inlineStr">
@@ -51180,7 +51196,7 @@
       </c>
       <c r="P685" s="8" t="inlineStr">
         <is>
-          <t>備料：因鍵盤絲印需要廠商印刷，齊料時間5/15,持續 Tracking 物料交期</t>
+          <t># 認證Risk  只有VN一筆訂單，排程 05/30， 認證06/10 ready 須請Weibu加快認證速度 PIC:Weibu</t>
         </is>
       </c>
     </row>
@@ -53898,7 +53914,7 @@
           <t>Modern A14 J1M</t>
         </is>
       </c>
-      <c r="D722" s="23" t="inlineStr">
+      <c r="D722" s="25" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -53951,12 +53967,12 @@
       </c>
       <c r="O722" s="4" t="inlineStr">
         <is>
-          <t>4/27 試產物料轉運微步，待物料到料後安排MVT試產，</t>
+          <t>4/27 試產物料轉運微步，預計5/7安排MVT試產</t>
         </is>
       </c>
       <c r="P722" s="4" t="inlineStr">
         <is>
-          <t>物料 1)WLAN ETA@7/17 , gap 32d 2)adaptor ETA@7/20,gap 35d ，2）AVAP ，微步暫未建立code，影響adaptor/電腦包/Mouse,需微步盡快建立Vendercode for備料，認證：需微步協助盡快安排C E Report在6/B ready,滿足6/E TTM</t>
+          <t># 物料  WLAN：(2K ETA 6/B ,8K 7/B ETA ,其餘6K  L/T 六個月) ADP ： 需pull-in到06/15  PIC:微步/PUR # 認證Risk      CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨 PIC:Weibu</t>
         </is>
       </c>
     </row>
@@ -53974,7 +53990,7 @@
           <t>Modern A16 J1M</t>
         </is>
       </c>
-      <c r="D723" s="23" t="inlineStr">
+      <c r="D723" s="25" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -54027,12 +54043,12 @@
       </c>
       <c r="O723" s="4" t="inlineStr">
         <is>
-          <t>4/24 試產物料轉運微步，待物料到料後安排MVT試產</t>
+          <t>4/27 試產物料轉運微步，預計5/7安排MVT試產</t>
         </is>
       </c>
       <c r="P723" s="4" t="inlineStr">
         <is>
-          <t>物料 1)WLAN ETA@7/17 , gap 32d 2)adaptor ETA@7/20,gap 35d ，2）AVAP ，微步暫未建立code，影響adaptor/電腦包/Mouse,需微步盡快建立Vendercode for備料，認證：需微步協助盡快安排C E Report在6/B ready,滿足6/E TTM</t>
+          <t># 物料  WLAN：(2K ETA 6/B ,8K 7/B ETA ,其餘6K  L/T 六個月) ADP ： 需pull-in到06/15  PIC:微步/PUR # 認證Risk      CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨 PIC:Weibu</t>
         </is>
       </c>
     </row>
@@ -55986,12 +56002,12 @@
       </c>
       <c r="N750" s="4" t="inlineStr">
         <is>
-          <t>2026/05/30</t>
+          <t>2026/05/28</t>
         </is>
       </c>
       <c r="O750" s="4" t="inlineStr">
         <is>
-          <t>1. ATS reschedule. SMT on 5/7, Assembly on 5/13.</t>
+          <t>1. ATS reschedule. SMT on 5/7, Assembly on 5/11, Customer Inspection on 5/21.</t>
         </is>
       </c>
       <c r="P750" s="4" t="inlineStr">
@@ -56014,7 +56030,7 @@
           <t>Venture 15 AI A2HMGO</t>
         </is>
       </c>
-      <c r="D751" s="18" t="inlineStr">
+      <c r="D751" s="24" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
@@ -56061,7 +56077,11 @@
           <t>2026/05/21</t>
         </is>
       </c>
-      <c r="O751" s="4" t="inlineStr"/>
+      <c r="O751" s="4" t="inlineStr">
+        <is>
+          <t>DQA 驗證中</t>
+        </is>
+      </c>
       <c r="P751" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -57182,9 +57202,9 @@
           <t>Venture 15 B3M</t>
         </is>
       </c>
-      <c r="D767" s="20" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D767" s="25" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E767" s="4" t="inlineStr">
@@ -57235,12 +57255,12 @@
       </c>
       <c r="O767" s="4" t="inlineStr">
         <is>
-          <t>預計4/27@0A layout start</t>
+          <t>0A layout中</t>
         </is>
       </c>
       <c r="P767" s="4" t="inlineStr">
         <is>
-          <t>1.Color Plan未定案影響開模,schedule待定案後確認</t>
+          <t>15T2 時程相當緊急, 組裝僅有一次MVT,之後就進入ATS,由於系列設計尚未定案，team member 目前無法確認開模與修模方向,且部分模具與 15T1/15T3 共用,仍需協調可挪用時程,請 ID/SPM 務必於 5/5 前完成定案.</t>
         </is>
       </c>
     </row>
@@ -57258,7 +57278,7 @@
           <t>Venture 17 AI A2HMGO</t>
         </is>
       </c>
-      <c r="D768" s="18" t="inlineStr">
+      <c r="D768" s="24" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
@@ -57292,7 +57312,7 @@
       </c>
       <c r="L768" s="4" t="inlineStr">
         <is>
-          <t>2026/04/24</t>
+          <t>2026/04/27</t>
         </is>
       </c>
       <c r="M768" s="4" t="inlineStr">
@@ -57307,7 +57327,7 @@
       </c>
       <c r="O768" s="4" t="inlineStr">
         <is>
-          <t>MVT 待上線</t>
+          <t>DQA 測試中</t>
         </is>
       </c>
       <c r="P768" s="4" t="inlineStr">
@@ -58510,7 +58530,7 @@
           <t>Venture 16 AI A2HMGO</t>
         </is>
       </c>
-      <c r="D785" s="18" t="inlineStr">
+      <c r="D785" s="24" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
@@ -58557,7 +58577,11 @@
           <t>2026/05/21</t>
         </is>
       </c>
-      <c r="O785" s="4" t="inlineStr"/>
+      <c r="O785" s="4" t="inlineStr">
+        <is>
+          <t>DQA 驗證中</t>
+        </is>
+      </c>
       <c r="P785" s="4" t="inlineStr">
         <is>
           <t>NA</t>
@@ -61014,7 +61038,7 @@
           <t>Modern 16S G3MG</t>
         </is>
       </c>
-      <c r="D819" s="24" t="inlineStr">
+      <c r="D819" s="19" t="inlineStr">
         <is>
           <t>ATS</t>
         </is>
@@ -61066,17 +61090,17 @@
       </c>
       <c r="N819" s="4" t="inlineStr">
         <is>
-          <t>2026/05/11</t>
+          <t>2026/05/13</t>
         </is>
       </c>
       <c r="O819" s="4" t="inlineStr">
         <is>
-          <t>1. Rebuild BIOS 103 to fix RPMC and abnormal shutdown issues.</t>
+          <t>1. 4/28客驗Fail, Compal重新提供對策後5/7做第二次客驗.</t>
         </is>
       </c>
       <c r="P819" s="4" t="inlineStr">
         <is>
-          <t>1. RPMC and abnormal shutdown issues happening in run-in process.</t>
+          <t>None.</t>
         </is>
       </c>
     </row>
@@ -61686,7 +61710,7 @@
           <t>Claw 8 EX AI+ CG3EM</t>
         </is>
       </c>
-      <c r="D828" s="18" t="inlineStr">
+      <c r="D828" s="24" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
@@ -61733,7 +61757,7 @@
       </c>
       <c r="M828" s="4" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
+          <t>2026/05/11</t>
         </is>
       </c>
       <c r="N828" s="4" t="inlineStr">
@@ -61743,12 +61767,12 @@
       </c>
       <c r="O828" s="4" t="inlineStr">
         <is>
-          <t>MVT DQA test4/15-4/29</t>
+          <t>MVT DQA test4/15-4/29，debug end@5/7</t>
         </is>
       </c>
       <c r="P828" s="4" t="inlineStr">
         <is>
-          <t>Gating  物料       1)Packing :包材落摔fail, Packing solution確定@4/27. 持續追蹤   NPI issue      1)Mura &gt; 100 Lux , waive申請      2) ME locK更新後不開機 .RD debugging.      3) 3C認證要到5/E,中國區出貨受影響</t>
+          <t>Gating  物料       1)Packing :三合一Packing圖面&amp;料號fix@4/30, target 5/12交料, 請採購追蹤交期中 NPI issue      1)Mura &gt; 100 Lux , waive申請      2) ME locK更新後不開機 .工廠修改指令驗證QS CPU pass, 5/6驗證MP CPU      3) 3C認證要到5/E,中國區出貨受影響</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update 周三 2026/05/06 10:06:54.05
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -51105,12 +51105,12 @@
       </c>
       <c r="M684" s="4" t="inlineStr">
         <is>
-          <t>2026/05/09</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="N684" s="4" t="inlineStr">
         <is>
-          <t>2026/05/21</t>
+          <t>2026/05/30</t>
         </is>
       </c>
       <c r="O684" s="4" t="inlineStr">
@@ -51120,7 +51120,7 @@
       </c>
       <c r="P684" s="4" t="inlineStr">
         <is>
-          <t>物料 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  認證  泰國 需業務push進口商提供認證資料,資料Ready後+3W PIC: Sales   馬來西亞 進口商WIFI 模組證書失效需盡快提供認證資料, 資料Ready後+5W PIC: Sale</t>
+          <t>1.物料: 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  2.認證: 泰國 需業務push進口商提供認證資料,資料Ready後+3W PIC: Sales   馬來西亞 進口商WIFI 模組證書失效需盡快提供認證資料, 資料Ready後+5W PIC: Sale</t>
         </is>
       </c>
     </row>
@@ -51196,7 +51196,7 @@
       </c>
       <c r="P685" s="8" t="inlineStr">
         <is>
-          <t># 認證Risk  只有VN一筆訂單，排程 05/30， 認證06/10 ready 須請Weibu加快認證速度 PIC:Weibu</t>
+          <t>1.物料: 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  2.認證:  只有VN一筆訂單，排程 05/30， 認證06/10 ready 須請Weibu加快認證速度 PIC:Weibu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update 周四 2026/05/07 13:20:24.77
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -30715,12 +30715,12 @@
       </c>
       <c r="O410" s="8" t="inlineStr">
         <is>
-          <t>暫定 5/20 ATS Assy, 5/30 2nd MP</t>
+          <t>預計5/20 ATS Assy 9S7-15TK11-040*100</t>
         </is>
       </c>
       <c r="P410" s="8" t="inlineStr">
         <is>
-          <t>4/30備料會議討論後暫定 5/20 ATS Assy, 5/30 2nd MP,最終 ATS 時程將依物料齊套狀況再行調整,目前已知缺料瓶頸為 KB shielding,已重新開 BTO,請 Vincent/Eva 協助通知業務儘速下單入系統,以利物管確認是否仍有其他缺料項目</t>
+          <t>工單剛入系統,KB shielding預計5/15進場,物管在確認是否還有其他缺料</t>
         </is>
       </c>
     </row>
@@ -30867,7 +30867,7 @@
       </c>
       <c r="O412" s="8" t="inlineStr">
         <is>
-          <t>同Cyborg A15 Max C1WG</t>
+          <t>預計5/20 C/R 9S7-15TK21-037*50</t>
         </is>
       </c>
       <c r="P412" s="8" t="inlineStr">
@@ -61757,12 +61757,12 @@
       </c>
       <c r="M828" s="4" t="inlineStr">
         <is>
-          <t>2026/05/18</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="N828" s="4" t="inlineStr">
         <is>
-          <t>2026/05/28</t>
+          <t>2026/05/26</t>
         </is>
       </c>
       <c r="O828" s="4" t="inlineStr">
@@ -61772,7 +61772,7 @@
       </c>
       <c r="P828" s="4" t="inlineStr">
         <is>
-          <t>1.物料：三合一Packing圖面&amp;料號fix@4/30, target 5/12交料, 包材廠商回復交期5/18,請採購追蹤交期中    2. 認證：3C認證測試battery cable輸出功率大於15W,待提供50cm延長線測試,中國區出貨受影響,拿到CCC認證時間TBD.</t>
+          <t>1.物料：三合一Packing圖面&amp;料號fix@4/30, target 5/12交料, 包材廠商回復交期5/11,請採購追蹤交期中,5/18更新進度    2. 認證：3C認證測試battery cable輸出功率大於15W,待提供50cm延長線測試,中國區出貨受影響,拿到CCC認證時間TBD.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update 2026/05/09 09:00
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -180,9 +180,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -553,7 +550,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -796,7 +793,7 @@
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
-          <t>1. AU*456Pcs1st MP 5/30出貨 2.VN *190Pcs  gating  認證ready 6/B , 3.KH *120Pcs  gating  Core 3 100U CPU缺料,5/11 出貨，5/17 到微步  4.TH *360Pcs gating  認證未ready，需進口商盡快提供資料，預抓5/15 資料ready，+3W 拿證6/5          5.CPU/B&amp;S物料 5/7已安排DHL快遞,微步確認需要5/10 到料才可滿足5/E 的MP規劃，持續追蹤, (PIC: PMC、微步） 6.KB: 4/24 weibu 收到訂單 安排對應鍵盤語言絲印，預計最快交期5/15，持續跟進微步 Pull-in 進度 (PIC: 微步) 7. 泰國認證：需業務推動進口商配合盡快處理認證所需資料，預抓5/15 資料ready，+3W 拿證6/5，，PIC sales/進口商            8. 馬來西亞認證：（Achieva）進口商WIFI 模組持證證書失效/進口商盡快提供認證所需資料，進口商 SIRIM 持證報告重辦 2 W～4W，资料ready後 + 5 周拿證，預計 7/M 拿證，PIC sales/進口商/weibu</t>
+          <t>同Cyborg 15 Black Edition A13UDO</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1165,7 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>1.NPI issue:Modern Standby 手動喚醒後,鍵盤無功能,fail rate:1/960,新版BIOS測試中,預計今天下午有結果 2.備料:KB shielding交期@5/15,KB交期採購物管push中</t>
+          <t>1.備料:KB shielding交期@5/15,KB物料 採購物管追蹤交期中</t>
         </is>
       </c>
     </row>
@@ -4818,9 +4815,9 @@
           <t>Modern A14 J1M</t>
         </is>
       </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -4871,12 +4868,12 @@
       </c>
       <c r="O59" s="4" t="inlineStr">
         <is>
-          <t>預計5/7安排MVT試產，RD Sample 5/11 ETD</t>
+          <t>預計5/7安排MVT試產，RD Sample 5/13 ETD</t>
         </is>
       </c>
       <c r="P59" s="4" t="inlineStr">
         <is>
-          <t>物料  WLAN：( 目標5/E ETA* 10K , 6K TBD , keep posting (PIC: 採購) ADP ： 需pull-in到06/15  PIC:微步/PUR ， 認證Risk      CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨 PIC:Weibu</t>
+          <t>1.物料 WLAN：5/28 ETA* 10K , 6K TBD ,  Adapter ：目標16K， 需pull-in到06/15  ETA 2.認證  CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨</t>
         </is>
       </c>
     </row>
@@ -4894,9 +4891,9 @@
           <t>Modern A16 J1M</t>
         </is>
       </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -4947,12 +4944,12 @@
       </c>
       <c r="O60" s="4" t="inlineStr">
         <is>
-          <t>預計5/7安排MVT試產，RD Sample 5/11 ETD</t>
+          <t>預計5/7安排MVT試產，RD Sample 5/13ETD</t>
         </is>
       </c>
       <c r="P60" s="4" t="inlineStr">
         <is>
-          <t>物料  WLAN：( 目標5/E ETA* 10K , 6K TBD , keep posting (PIC: 採購) ADP ： 需pull-in到06/15  PIC:微步/PUR ， 認證Risk      CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨 PIC:Weibu</t>
+          <t>1.物料 WLAN：5/28 ETA* 10K , 6K TBD ,  Adapter ：目標16K， 需pull-in到06/15  ETA 2.認證  CE需加急處理, 06/06 ready 才能meet 06/30 PH出貨</t>
         </is>
       </c>
     </row>
@@ -5050,9 +5047,9 @@
           <t>Venture 15 AI A2HMGO</t>
         </is>
       </c>
-      <c r="D62" s="12" t="inlineStr">
-        <is>
-          <t>MVT</t>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -5099,12 +5096,12 @@
       </c>
       <c r="O62" s="4" t="inlineStr">
         <is>
-          <t>DQA測試中</t>
+          <t>等業務訂單安排ATS</t>
         </is>
       </c>
       <c r="P62" s="4" t="inlineStr">
         <is>
-          <t>1. Schedule: DQA預計5/8測試完成,Schedule暫不影響,ATS待業務正式下單後確認上線時間</t>
+          <t>1. Schedule: 等業務訂單安排ATS</t>
         </is>
       </c>
     </row>
@@ -5318,17 +5315,17 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>17U1</t>
+          <t>2611</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Venture 17 AI A2HMGO</t>
-        </is>
-      </c>
-      <c r="D66" s="12" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Venture 16 AI A2HMGO</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -5343,7 +5340,7 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>顧曉琴</t>
+          <t>李文欽</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -5360,7 +5357,7 @@
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>2026/04/27</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
@@ -5375,12 +5372,12 @@
       </c>
       <c r="O66" s="4" t="inlineStr">
         <is>
-          <t>DQA 測試中</t>
+          <t>等業務訂單安排ATS</t>
         </is>
       </c>
       <c r="P66" s="4" t="inlineStr">
         <is>
-          <t>1. Schedule: DQA預計5/8測試完成,Schedule暫不影響,ATS待業務正式下單後確認上線時間</t>
+          <t>1. schedule: 等業務訂單安排ATS</t>
         </is>
       </c>
     </row>
@@ -5390,17 +5387,17 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>17U1</t>
+          <t>2611</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>VenturePro 17 AI A2HUDXG</t>
+          <t>VenturePro 16 AI A2HUDXG</t>
         </is>
       </c>
       <c r="D67" s="20" t="inlineStr">
         <is>
-          <t>ATS-</t>
+          <t>BTO-</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -5415,44 +5412,44 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>顧曉琴</t>
+          <t>李文欽</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>2025/05/29</t>
+          <t>2025/02/14</t>
         </is>
       </c>
       <c r="I67" s="8" t="inlineStr"/>
       <c r="J67" s="8" t="inlineStr"/>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>2025/06/09</t>
+          <t>2025/03/24</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr">
         <is>
+          <t>2025/03/21</t>
+        </is>
+      </c>
+      <c r="M67" s="8" t="inlineStr">
+        <is>
+          <t>2025/05/26</t>
+        </is>
+      </c>
+      <c r="N67" s="8" t="inlineStr">
+        <is>
           <t>2025/06/06</t>
         </is>
       </c>
-      <c r="M67" s="8" t="inlineStr">
-        <is>
-          <t>2025/07/07</t>
-        </is>
-      </c>
-      <c r="N67" s="8" t="inlineStr">
-        <is>
-          <t>2025/07/10</t>
-        </is>
-      </c>
       <c r="O67" s="8" t="inlineStr">
         <is>
-          <t>BTO已開,無業務訂單</t>
+          <t>-105</t>
         </is>
       </c>
       <c r="P67" s="8" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1. GPU缺料 2. 原US訂單無法上線改ATS訂單 3. FHD camera 卻料</t>
         </is>
       </c>
     </row>
@@ -5462,12 +5459,12 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>17U1</t>
+          <t>2611</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>VenturePro 17 AI A2HVEG</t>
+          <t>VenturePro 16 AI A2HVEG</t>
         </is>
       </c>
       <c r="D68" s="15" t="inlineStr">
@@ -5487,112 +5484,124 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>顧曉琴</t>
+          <t>李文欽</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>2025/05/29</t>
+          <t>2025/02/14</t>
         </is>
       </c>
       <c r="I68" s="8" t="inlineStr"/>
       <c r="J68" s="8" t="inlineStr"/>
       <c r="K68" s="8" t="inlineStr">
         <is>
-          <t>2025/06/09</t>
+          <t>2025/03/24</t>
         </is>
       </c>
       <c r="L68" s="8" t="inlineStr">
         <is>
+          <t>2025/03/21</t>
+        </is>
+      </c>
+      <c r="M68" s="8" t="inlineStr">
+        <is>
+          <t>2025/05/26</t>
+        </is>
+      </c>
+      <c r="N68" s="8" t="inlineStr">
+        <is>
           <t>2025/06/06</t>
         </is>
       </c>
-      <c r="M68" s="8" t="inlineStr">
-        <is>
-          <t>2025/07/07</t>
-        </is>
-      </c>
-      <c r="N68" s="8" t="inlineStr">
-        <is>
-          <t>2025/07/12</t>
-        </is>
-      </c>
       <c r="O68" s="8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-105</t>
         </is>
       </c>
       <c r="P68" s="8" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" hidden="1" outlineLevel="1">
-      <c r="A69" s="6" t="n">
+          <t>1. GPU缺料 2. 原US訂單無法上線改ATS訂單 3. FHD camera 卻料</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="7" t="inlineStr">
-        <is>
-          <t>17U1</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>VenturePro 17 AI A2HVEG</t>
-        </is>
-      </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>ARL-H 45W</t>
-        </is>
-      </c>
-      <c r="F69" s="8" t="inlineStr">
-        <is>
-          <t>RTX 4050 (35W+10W)/ GDDR6 6GB</t>
-        </is>
-      </c>
-      <c r="G69" s="8" t="inlineStr">
-        <is>
-          <t>顧曉琴</t>
-        </is>
-      </c>
-      <c r="H69" s="8" t="inlineStr">
-        <is>
-          <t>2025/05/29</t>
-        </is>
-      </c>
-      <c r="I69" s="8" t="inlineStr"/>
-      <c r="J69" s="8" t="inlineStr"/>
-      <c r="K69" s="8" t="inlineStr">
-        <is>
-          <t>2025/02/06</t>
-        </is>
-      </c>
-      <c r="L69" s="8" t="inlineStr">
-        <is>
-          <t>2025/03/10</t>
-        </is>
-      </c>
-      <c r="M69" s="8" t="inlineStr">
-        <is>
-          <t>2025/04/01</t>
-        </is>
-      </c>
-      <c r="N69" s="8" t="inlineStr">
-        <is>
-          <t>2025/04/15</t>
-        </is>
-      </c>
-      <c r="O69" s="8" t="inlineStr"/>
-      <c r="P69" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>26U3</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Modern 16S G3MG</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>ATS</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>林耀慶</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>2025/10/01</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>2025/11/17</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>2025/12/23</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>2026/02/03</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>2026/02/26</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/08</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/13</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>1. DQA客驗進行中. 2. QA客驗於5/8開始.</t>
+        </is>
+      </c>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
         </is>
       </c>
     </row>
@@ -5602,12 +5611,12 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>2611</t>
+          <t>1T91</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Venture 16 AI A2HMGO</t>
+          <t>Claw 8 EX AI+ CG3EM</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -5617,54 +5626,62 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>ARL-H 45W</t>
+          <t>PTL-H 25W</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Intel® Arc™ Graphics</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>李文欽</t>
+          <t>楊淑賢</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>2026/04/21</t>
-        </is>
-      </c>
-      <c r="I70" s="4" t="inlineStr"/>
-      <c r="J70" s="4" t="inlineStr"/>
+          <t>2025/11/06</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>2025/12/16</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>2026/01/31</t>
+        </is>
+      </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>2026/04/27</t>
+          <t>2026/04/02</t>
         </is>
       </c>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>2026/04/24</t>
+          <t>2026/04/09</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr">
         <is>
-          <t>2026/05/09</t>
+          <t>2026/05/14</t>
         </is>
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>2026/05/21</t>
+          <t>2026/05/26</t>
         </is>
       </c>
       <c r="O70" s="4" t="inlineStr">
         <is>
-          <t>DQA 驗證中</t>
+          <t>ATS SMT預抓5/14, ASSY 5/15</t>
         </is>
       </c>
       <c r="P70" s="4" t="inlineStr">
         <is>
-          <t>1. Schedule: DQA預計5/8測試完成,Schedule暫不影響,ATS待業務正式下單後確認上線時間</t>
+          <t>1.物料：三合一包材包材廠商回復交期5/18,請採購追蹤交期中 2. 認證：3C認證測試battery cable輸出功率大於15W,待提供50cm延長線測試;機構殼燃燒測試fail,中國區出貨受影響,拿到CCC認證時間預計6月初.</t>
         </is>
       </c>
     </row>
@@ -5674,69 +5691,65 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>2611</t>
+          <t>1T91</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>VenturePro 16 AI A2HUDXG</t>
-        </is>
-      </c>
-      <c r="D71" s="21" t="inlineStr">
-        <is>
-          <t>BTO-</t>
+          <t>Claw 8 EX AI+ CG3EM Launch Pack</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>ARL-H 45W</t>
+          <t>PTL-H 25W</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>RTX 3050 (35W+10W)/ GDDR6 6GB</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>李文欽</t>
+          <t>楊淑賢</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>2025/02/14</t>
+          <t>2025/11/06</t>
         </is>
       </c>
       <c r="I71" s="8" t="inlineStr"/>
       <c r="J71" s="8" t="inlineStr"/>
-      <c r="K71" s="8" t="inlineStr">
-        <is>
-          <t>2025/03/24</t>
-        </is>
-      </c>
+      <c r="K71" s="8" t="inlineStr"/>
       <c r="L71" s="8" t="inlineStr">
         <is>
-          <t>2025/03/21</t>
+          <t>2026/04/09</t>
         </is>
       </c>
       <c r="M71" s="8" t="inlineStr">
         <is>
-          <t>2025/05/26</t>
+          <t>2026/05/14</t>
         </is>
       </c>
       <c r="N71" s="8" t="inlineStr">
         <is>
-          <t>2025/06/06</t>
+          <t>2026/05/26</t>
         </is>
       </c>
       <c r="O71" s="8" t="inlineStr">
         <is>
-          <t>-105</t>
+          <t>大禮包包材follow 12XE</t>
         </is>
       </c>
       <c r="P71" s="8" t="inlineStr">
         <is>
-          <t>1. GPU缺料 2. 原US訂單無法上線改ATS訂單 3. FHD camera 卻料</t>
+          <t>follow 12XE</t>
         </is>
       </c>
     </row>
@@ -5746,382 +5759,82 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>2611</t>
+          <t>1T91</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>VenturePro 16 AI A2HVEG</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>MP</t>
+          <t>Claw 8 EX AI+ CG3M</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="inlineStr">
+        <is>
+          <t>BTO-</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>ARL-H 45W</t>
+          <t>PTL-H 25W</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>RTX 4050 (35W+10W)/ GDDR6 6GB</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>李文欽</t>
+          <t>楊淑賢</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>2025/02/14</t>
-        </is>
-      </c>
-      <c r="I72" s="8" t="inlineStr"/>
-      <c r="J72" s="8" t="inlineStr"/>
+          <t>2025/11/06</t>
+        </is>
+      </c>
+      <c r="I72" s="8" t="inlineStr">
+        <is>
+          <t>2025/12/16</t>
+        </is>
+      </c>
+      <c r="J72" s="8" t="inlineStr">
+        <is>
+          <t>2026/01/31</t>
+        </is>
+      </c>
       <c r="K72" s="8" t="inlineStr">
         <is>
-          <t>2025/03/24</t>
+          <t>2026/04/02</t>
         </is>
       </c>
       <c r="L72" s="8" t="inlineStr">
         <is>
-          <t>2025/03/21</t>
+          <t>2026/04/08</t>
         </is>
       </c>
       <c r="M72" s="8" t="inlineStr">
         <is>
-          <t>2025/05/26</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="N72" s="8" t="inlineStr">
         <is>
-          <t>2025/06/06</t>
+          <t>2026/05/23</t>
         </is>
       </c>
       <c r="O72" s="8" t="inlineStr">
         <is>
-          <t>-105</t>
+          <t>暫無業務需求，未開放BTO</t>
         </is>
       </c>
       <c r="P72" s="8" t="inlineStr">
         <is>
-          <t>1. GPU缺料 2. 原US訂單無法上線改ATS訂單 3. FHD camera 卻料</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>26U3</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Modern 16S G3MG</t>
-        </is>
-      </c>
-      <c r="D73" s="10" t="inlineStr">
-        <is>
-          <t>ATS</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>WCL 25W</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Intel® graphics</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>林耀慶</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>2025/10/01</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>2025/11/17</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="inlineStr">
-        <is>
-          <t>2025/12/23</t>
-        </is>
-      </c>
-      <c r="K73" s="4" t="inlineStr">
-        <is>
-          <t>2026/02/03</t>
-        </is>
-      </c>
-      <c r="L73" s="4" t="inlineStr">
-        <is>
-          <t>2026/02/26</t>
-        </is>
-      </c>
-      <c r="M73" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/08</t>
-        </is>
-      </c>
-      <c r="N73" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/13</t>
-        </is>
-      </c>
-      <c r="O73" s="4" t="inlineStr">
-        <is>
-          <t>1. DQA客驗進行中. 2. QA客驗於5/8開始.</t>
-        </is>
-      </c>
-      <c r="P73" s="4" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>1T91</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>Claw 8 EX AI+ CG3EM</t>
-        </is>
-      </c>
-      <c r="D74" s="12" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>PTL-H 25W</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G74" s="4" t="inlineStr">
-        <is>
-          <t>楊淑賢</t>
-        </is>
-      </c>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>2025/11/06</t>
-        </is>
-      </c>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>2025/12/16</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>2026/01/31</t>
-        </is>
-      </c>
-      <c r="K74" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/02</t>
-        </is>
-      </c>
-      <c r="L74" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/09</t>
-        </is>
-      </c>
-      <c r="M74" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/15</t>
-        </is>
-      </c>
-      <c r="N74" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/26</t>
-        </is>
-      </c>
-      <c r="O74" s="4" t="inlineStr">
-        <is>
-          <t>MVT DQA test4/15-4/29，debug end@5/7</t>
-        </is>
-      </c>
-      <c r="P74" s="4" t="inlineStr">
-        <is>
-          <t>1.物料：三合一包材包材廠商回復交期5/18,請採購追蹤交期中 2. 認證：3C認證測試battery cable輸出功率大於15W,待提供50cm延長線測試;機構殼燃燒測試fail,中國區出貨受影響,拿到CCC認證時間預計6月初.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1">
-      <c r="A75" s="6" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>1T91</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>Claw 8 EX AI+ CG3EM Launch Pack</t>
-        </is>
-      </c>
-      <c r="D75" s="13" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>PTL-H 25W</t>
-        </is>
-      </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G75" s="8" t="inlineStr">
-        <is>
-          <t>楊淑賢</t>
-        </is>
-      </c>
-      <c r="H75" s="8" t="inlineStr">
-        <is>
-          <t>2025/11/06</t>
-        </is>
-      </c>
-      <c r="I75" s="8" t="inlineStr"/>
-      <c r="J75" s="8" t="inlineStr"/>
-      <c r="K75" s="8" t="inlineStr"/>
-      <c r="L75" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/09</t>
-        </is>
-      </c>
-      <c r="M75" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="N75" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/26</t>
-        </is>
-      </c>
-      <c r="O75" s="8" t="inlineStr">
-        <is>
-          <t>大禮包包材follow 12XE</t>
-        </is>
-      </c>
-      <c r="P75" s="8" t="inlineStr">
-        <is>
-          <t>follow 12XE</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" hidden="1" outlineLevel="1">
-      <c r="A76" s="6" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
-        <is>
-          <t>1T91</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>Claw 8 EX AI+ CG3M</t>
-        </is>
-      </c>
-      <c r="D76" s="21" t="inlineStr">
-        <is>
-          <t>BTO-</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>PTL-H 25W</t>
-        </is>
-      </c>
-      <c r="F76" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G76" s="8" t="inlineStr">
-        <is>
-          <t>楊淑賢</t>
-        </is>
-      </c>
-      <c r="H76" s="8" t="inlineStr">
-        <is>
-          <t>2025/11/06</t>
-        </is>
-      </c>
-      <c r="I76" s="8" t="inlineStr">
-        <is>
-          <t>2025/12/16</t>
-        </is>
-      </c>
-      <c r="J76" s="8" t="inlineStr">
-        <is>
-          <t>2026/01/31</t>
-        </is>
-      </c>
-      <c r="K76" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/02</t>
-        </is>
-      </c>
-      <c r="L76" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/08</t>
-        </is>
-      </c>
-      <c r="M76" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="N76" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/23</t>
-        </is>
-      </c>
-      <c r="O76" s="8" t="inlineStr">
-        <is>
-          <t>暫無業務需求，未開放BTO</t>
-        </is>
-      </c>
-      <c r="P76" s="8" t="inlineStr">
-        <is>
           <t>follow 12xe</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P76"/>
+  <autoFilter ref="A1:P72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto update 2026/05/12 08:46
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -5847,12 +5847,12 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>14V2</t>
+          <t>14T2</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Modern 14 H1M</t>
+          <t>Prestige 14 Flip AI+ Rhône</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -5862,206 +5862,206 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>RPL-U refresh	 25W</t>
+          <t>PTL-H 30W</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱芳芳</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>2026/01/04</t>
-        </is>
-      </c>
+          <t>2026/04/13</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr"/>
       <c r="J73" s="4" t="inlineStr"/>
       <c r="K73" s="4" t="inlineStr">
         <is>
+          <t>2026/05/10</t>
+        </is>
+      </c>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/26</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/22</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/30</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>MVT SMT:5/10, ASSY:5/15</t>
+        </is>
+      </c>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>14V2</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Commercial 14 C1M</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>RPL-U refresh	 25W</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>2025/11/14</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>2026/01/04</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr"/>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
           <t>2026/01/14</t>
         </is>
       </c>
-      <c r="L73" s="4" t="inlineStr">
+      <c r="L74" s="4" t="inlineStr">
         <is>
           <t>2026/03/16</t>
         </is>
       </c>
-      <c r="M73" s="4" t="inlineStr">
+      <c r="M74" s="4" t="inlineStr">
         <is>
           <t>2026/05/15</t>
         </is>
       </c>
-      <c r="N73" s="4" t="inlineStr">
+      <c r="N74" s="4" t="inlineStr">
         <is>
           <t>2026/05/30</t>
         </is>
       </c>
-      <c r="O73" s="4" t="inlineStr">
+      <c r="O74" s="4" t="inlineStr">
+        <is>
+          <t>MVT debug中，Base  on 物料Ready時間安排ATS</t>
+        </is>
+      </c>
+      <c r="P74" s="4" t="inlineStr">
+        <is>
+          <t>1.物料: 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  2.認證:  只有VN一筆訂單，排程 05/30， 認證06/10 ready 須請Weibu加快認證速度 PIC:Weibu</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="A75" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>14V2</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Modern 14 H1M</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>RPL-U refresh	 25W</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>2025/11/14</t>
+        </is>
+      </c>
+      <c r="I75" s="8" t="inlineStr">
+        <is>
+          <t>2026/01/04</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr"/>
+      <c r="K75" s="8" t="inlineStr">
+        <is>
+          <t>2026/01/14</t>
+        </is>
+      </c>
+      <c r="L75" s="8" t="inlineStr">
+        <is>
+          <t>2026/03/16</t>
+        </is>
+      </c>
+      <c r="M75" s="8" t="inlineStr">
+        <is>
+          <t>2026/05/15</t>
+        </is>
+      </c>
+      <c r="N75" s="8" t="inlineStr">
+        <is>
+          <t>2026/05/30</t>
+        </is>
+      </c>
+      <c r="O75" s="8" t="inlineStr">
         <is>
           <t>MVT debug中，,Base on 物料Ready時間安排 ATS上線</t>
         </is>
       </c>
-      <c r="P73" s="4" t="inlineStr">
+      <c r="P75" s="8" t="inlineStr">
         <is>
           <t>1.物料: 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  2.認證: 抓5/15 資料ready，+3W 拿證6/5 PIC: Sales   馬來西亞 進口商WIFI 模組證書失效&amp;提供認證資料, 預計7/M拿證PIC: Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" hidden="1" outlineLevel="1">
-      <c r="A74" s="6" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>14V2</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>Commercial 14 C1M</t>
-        </is>
-      </c>
-      <c r="D74" s="13" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>RPL-U refresh	 25W</t>
-        </is>
-      </c>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G74" s="8" t="inlineStr">
-        <is>
-          <t>杜晨光</t>
-        </is>
-      </c>
-      <c r="H74" s="8" t="inlineStr">
-        <is>
-          <t>2025/11/14</t>
-        </is>
-      </c>
-      <c r="I74" s="8" t="inlineStr">
-        <is>
-          <t>2026/01/04</t>
-        </is>
-      </c>
-      <c r="J74" s="8" t="inlineStr"/>
-      <c r="K74" s="8" t="inlineStr">
-        <is>
-          <t>2026/01/14</t>
-        </is>
-      </c>
-      <c r="L74" s="8" t="inlineStr">
-        <is>
-          <t>2026/03/16</t>
-        </is>
-      </c>
-      <c r="M74" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/15</t>
-        </is>
-      </c>
-      <c r="N74" s="8" t="inlineStr">
-        <is>
-          <t>2026/05/30</t>
-        </is>
-      </c>
-      <c r="O74" s="8" t="inlineStr">
-        <is>
-          <t>MVT debug中，Base  on 物料Ready時間安排ATS</t>
-        </is>
-      </c>
-      <c r="P74" s="8" t="inlineStr">
-        <is>
-          <t>1.物料: 需05/15齊料, 才能meet 05/30 TTM (Risk物料 CPU/ADP/KB) PIC:PMC/PUR  2.認證:  只有VN一筆訂單，排程 05/30， 認證06/10 ready 須請Weibu加快認證速度 PIC:Weibu</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>14T2</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 14 Flip AI+ Rhône</t>
-        </is>
-      </c>
-      <c r="D75" s="12" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>PTL-H 30W</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/13</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr"/>
-      <c r="J75" s="4" t="inlineStr"/>
-      <c r="K75" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/10</t>
-        </is>
-      </c>
-      <c r="L75" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/26</t>
-        </is>
-      </c>
-      <c r="M75" s="4" t="inlineStr">
-        <is>
-          <t>2026/06/22</t>
-        </is>
-      </c>
-      <c r="N75" s="4" t="inlineStr">
-        <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="O75" s="4" t="inlineStr">
-        <is>
-          <t>MVT SMT:5/10, ASSY:5/15</t>
-        </is>
-      </c>
-      <c r="P75" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>